<commit_message>
Rebuild the issued sign-off sets BRD-01, BRD-03, BRD-11, BRD-13 (files 00 to 05/06) and the Drop 0 closure set v2.0 with the business wording and Who signs what; the placement channel message as the platform shows it; the legacy record status list in the Drop 0 inputs map
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/03_BIBS_Signoff_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/03_BIBS_Signoff_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -27,7 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_lists" sheetId="18" state="hidden" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$141</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to review'!$A$4:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to review'!$4:$4</definedName>
@@ -57,7 +57,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="14">'Meeting minutes'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Version history'!$A$4:$E$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'Version history'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Sign-off certificate'!$A$4:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Sign-off certificate'!$A$4:$J$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'Sign-off certificate'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="D35" s="14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
@@ -25934,17 +25934,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -25970,44 +25972,56 @@
       <c r="F3" s="23" t="n"/>
       <c r="G3" s="23" t="n"/>
       <c r="H3" s="23" t="n"/>
+      <c r="I3" s="23" t="n"/>
+      <c r="J3" s="23" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Signs for</t>
-        </is>
-      </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
+          <t>Confirms</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>On the BRD approval sheet</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="F4" s="24" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="G4" s="24" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -26016,194 +26030,402 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Product Owner, Marketing Business System</t>
+          <t>Prepared by</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>BDOI</t>
+          <t>iorta TechNXT project team: Project Manager, Business Analysis, test lead</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Business owner: the whole set</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="12" t="n"/>
+          <t>iorta TechNXT</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>The set is complete and consistent as issued, traced to the BRD and to the screens; every comment is answered in the comments log</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Added for this set (author of the FRS set)</t>
+        </is>
+      </c>
       <c r="F5" s="12" t="n"/>
       <c r="G5" s="12" t="n"/>
-      <c r="H5" s="25" t="n"/>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="25" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Head, Marketing Business Services and System Support</t>
+          <t>Prepared by</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>BDOI</t>
+          <t>Business Analyst, Enterprise Services Group - Business Project Services (BPS)</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Set-up, versions, masters, incentive criteria and the configuration inputs</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="12" t="n"/>
+          <t>BDO Unibank ESG</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>The set states the BRD requirements as written; every departure is listed in the proposed rules and clarifications</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Prepared by (p.34, p.8)</t>
+        </is>
+      </c>
       <c r="F6" s="12" t="n"/>
       <c r="G6" s="12" t="n"/>
-      <c r="H6" s="25" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Head, Technical Support Unit</t>
+          <t>Input provided by</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
+          <t>Technical Support Unit (TSU), BU representatives</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
           <t>BDOI</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Package requests, negotiation, requirements, advisories and expiry</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="12" t="n"/>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>The package request, negotiation, requirements, advisory and expiry screens match the business input</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Input provided by (p.34, p.8)</t>
+        </is>
+      </c>
       <c r="F7" s="12" t="n"/>
       <c r="G7" s="12" t="n"/>
-      <c r="H7" s="25" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Head, Retail Marketing</t>
+          <t>Input provided by</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
+          <t>Marketing Business System (MBS), BU representatives</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
           <t>BDOI</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Package requests, approvals and pricing screens</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>The set-up, version, master and incentive screens and the configuration inputs match the business input</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Input provided by and Reviewed by (p.34, p.8)</t>
+        </is>
+      </c>
       <c r="F8" s="12" t="n"/>
       <c r="G8" s="12" t="n"/>
-      <c r="H8" s="25" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="25" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Head, Comptrollership</t>
+          <t>Reviewed by</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>BDOI</t>
+          <t>Program Manager, Enterprise Services Group - Business Project Services (BPS)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Finance: rates and taxes, commission rates, incentive criteria</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
+          <t>BDO Unibank ESG</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Traceability of every BRD requirement to the set and completeness of the set</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed by (p.34, p.9)</t>
+        </is>
+      </c>
       <c r="F9" s="12" t="n"/>
       <c r="G9" s="12" t="n"/>
-      <c r="H9" s="25" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="25" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Head, BDOI IT</t>
+          <t>Reviewed by</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
+          <t>BDOI Information Technology Group (BDOI IT)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
           <t>BDOI</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>BDOI IT: interfaces, user access and menus</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Interfaces, user access and menus, and the Technical Specification (a separate document); not the business screens</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Added for this set</t>
+        </is>
+      </c>
       <c r="F10" s="12" t="n"/>
       <c r="G10" s="12" t="n"/>
-      <c r="H10" s="25" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="25" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Program Manager, Business Project Services</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>BDO Unibank ESG</t>
+          <t>Product Owner, Marketing Business System</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Traceability to the BRD</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="12" t="n"/>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Owns the set and approves all of its contents</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.34, p.9)</t>
+        </is>
+      </c>
       <c r="F11" s="12" t="n"/>
       <c r="G11" s="12" t="n"/>
-      <c r="H11" s="25" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="25" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT</t>
+          <t>Unit Head - Claims, Analytics, Risk Management, Reinsurance and Technical Underwriting</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Delivery of the set as signed</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>The TSU part: package requests, negotiation, requirements, advisories and expiry</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.35, p.9)</t>
+        </is>
+      </c>
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="12" t="n"/>
-      <c r="H12" s="25" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Unit Head - Combank and Corbank</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Package requests, approvals and pricing for Combank and Corbank</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.35, p.9)</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="25" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Head - Retail Marketing</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Package requests, approvals and pricing for Retail Marketing</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.35, p.9)</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="25" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Head - Corporate and Retail Marketing</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Package requests, approvals and pricing for Corporate Marketing</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.35)</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="25" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Head - Comptrollership</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>BDOI</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Rates and taxes, commission rates and incentive criteria</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Approved by (p.35; marked not required on the addendum, p.9)</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="25" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H12"/>
+  <autoFilter ref="A4:J16"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:H512">
+  <conditionalFormatting sqref="A5:J516">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E512" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Decision" error="Choose a value from the list (Decision)." type="list">
+    <dataValidation sqref="G5:G516" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Decision" error="Choose a value from the list (Decision)." type="list">
       <formula1>'_lists'!$I$1:$I$3</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Review date" error="Enter a date (dd-mmm-yyyy)." type="date" operator="greaterThan">
+    <dataValidation sqref="J5:J5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Review date" error="Enter a date (dd-mmm-yyyy)." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -26396,7 +26618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D139"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28767,12 +28989,12 @@
       </c>
       <c r="B132" s="21" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="C132" s="14" t="inlineStr">
         <is>
-          <t>Signatory role</t>
+          <t>Prepared by, Input provided by, Reviewed by or Approved by, as on the BRD approval sheet</t>
         </is>
       </c>
       <c r="D132" s="14" t="inlineStr"/>
@@ -28785,12 +29007,12 @@
       </c>
       <c r="B133" s="20" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C133" s="12" t="inlineStr">
         <is>
-          <t>Organisation</t>
+          <t>Signatory role</t>
         </is>
       </c>
       <c r="D133" s="12" t="inlineStr"/>
@@ -28803,12 +29025,12 @@
       </c>
       <c r="B134" s="21" t="inlineStr">
         <is>
-          <t>Signs for</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="C134" s="14" t="inlineStr">
         <is>
-          <t>Part of the set the signatory confirms</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="D134" s="14" t="inlineStr"/>
@@ -28821,12 +29043,12 @@
       </c>
       <c r="B135" s="20" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Confirms</t>
         </is>
       </c>
       <c r="C135" s="12" t="inlineStr">
         <is>
-          <t>Name of the signatory</t>
+          <t>What the signatory confirms by signing</t>
         </is>
       </c>
       <c r="D135" s="12" t="inlineStr"/>
@@ -28839,19 +29061,15 @@
       </c>
       <c r="B136" s="21" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>On the BRD approval sheet</t>
         </is>
       </c>
       <c r="C136" s="14" t="inlineStr">
         <is>
-          <t>Approved, Approved with comments or Not approved</t>
-        </is>
-      </c>
-      <c r="D136" s="14" t="inlineStr">
-        <is>
-          <t>Approved, Approved with comments, Not approved</t>
-        </is>
-      </c>
+          <t>Where the role signs the BRD (BRD-3 approval sheets: main BRD p.34-35; Workshop Addendum p.8-9)</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
@@ -28861,12 +29079,12 @@
       </c>
       <c r="B137" s="20" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C137" s="12" t="inlineStr">
         <is>
-          <t>Conditions of the approval</t>
+          <t>Name of the signatory</t>
         </is>
       </c>
       <c r="D137" s="12" t="inlineStr"/>
@@ -28879,15 +29097,19 @@
       </c>
       <c r="B138" s="21" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C138" s="14" t="inlineStr">
         <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="D138" s="14" t="inlineStr"/>
+          <t>Approved, Approved with comments or Not approved</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Approved, Approved with comments, Not approved</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
@@ -28897,18 +29119,54 @@
       </c>
       <c r="B139" s="20" t="inlineStr">
         <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="C139" s="12" t="inlineStr">
+        <is>
+          <t>Conditions of the approval</t>
+        </is>
+      </c>
+      <c r="D139" s="12" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="inlineStr">
+        <is>
+          <t>Sign-off certificate</t>
+        </is>
+      </c>
+      <c r="B140" s="21" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C140" s="14" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="D140" s="14" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="12" t="inlineStr">
+        <is>
+          <t>Sign-off certificate</t>
+        </is>
+      </c>
+      <c r="B141" s="20" t="inlineStr">
+        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C139" s="12" t="inlineStr">
+      <c r="C141" s="12" t="inlineStr">
         <is>
           <t>Date of the decision</t>
         </is>
       </c>
-      <c r="D139" s="12" t="inlineStr"/>
+      <c r="D141" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D139"/>
+  <autoFilter ref="A4:D141"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -48387,7 +48645,7 @@
       </c>
       <c r="L244" s="12" t="inlineStr">
         <is>
-          <t>Valid JSON</t>
+          <t>Name and value pairs as in the example</t>
         </is>
       </c>
       <c r="M244" s="12" t="inlineStr">
@@ -68203,7 +68461,7 @@
       </c>
       <c r="G197" s="12" t="inlineStr">
         <is>
-          <t>Enter the rule parameters as valid JSON, for example {"minimumPremium": 5000}.</t>
+          <t>Enter the rule parameters as name and value pairs in braces, as in the example {"minimumPremium": 5000}.</t>
         </is>
       </c>
       <c r="H197" s="12" t="n"/>

</xml_diff>